<commit_message>
new results and new hh experiments
</commit_message>
<xml_diff>
--- a/benchmarking/analysis/averages.xlsx
+++ b/benchmarking/analysis/averages.xlsx
@@ -8,11 +8,12 @@
     <sheet state="visible" name="exp1-tall" sheetId="3" r:id="rId7"/>
     <sheet state="visible" name="exp-compact-wide" sheetId="4" r:id="rId8"/>
     <sheet state="visible" name="exp-compact-tall" sheetId="5" r:id="rId9"/>
-    <sheet state="visible" name="comparison" sheetId="6" r:id="rId10"/>
-    <sheet state="visible" name="exp-dl-wide" sheetId="7" r:id="rId11"/>
-    <sheet state="visible" name="exp-dl-tall" sheetId="8" r:id="rId12"/>
-    <sheet state="visible" name="exp-map-wide" sheetId="9" r:id="rId13"/>
-    <sheet state="visible" name="exp-map-tall" sheetId="10" r:id="rId14"/>
+    <sheet state="visible" name="exp-mcompact-wide" sheetId="6" r:id="rId10"/>
+    <sheet state="visible" name="comparison" sheetId="7" r:id="rId11"/>
+    <sheet state="visible" name="exp-dl-wide" sheetId="8" r:id="rId12"/>
+    <sheet state="visible" name="exp-dl-tall" sheetId="9" r:id="rId13"/>
+    <sheet state="visible" name="exp-map-wide" sheetId="10" r:id="rId14"/>
+    <sheet state="visible" name="exp-map-tall" sheetId="11" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="56">
   <si>
     <t>trains</t>
   </si>
@@ -83,6 +84,15 @@
   </si>
   <si>
     <t xml:space="preserve">drive-map-hypergraph					</t>
+  </si>
+  <si>
+    <t>more-compact-edge-functions</t>
+  </si>
+  <si>
+    <t>more-compact-subnodes</t>
+  </si>
+  <si>
+    <t>more-compact-hypergraph</t>
   </si>
   <si>
     <t>MAPF</t>
@@ -456,11 +466,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="728059248"/>
-        <c:axId val="1970567130"/>
+        <c:axId val="1327703412"/>
+        <c:axId val="1935581107"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="728059248"/>
+        <c:axId val="1327703412"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -512,10 +522,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1970567130"/>
+        <c:crossAx val="1935581107"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1970567130"/>
+        <c:axId val="1935581107"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -590,7 +600,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="728059248"/>
+        <c:crossAx val="1327703412"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -624,6 +634,10 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
@@ -641,6 +655,10 @@
 </file>
 
 <file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
   <xdr:oneCellAnchor>
     <xdr:from>
@@ -668,10 +686,6 @@
     <xdr:clientData fLocksWithSheet="0"/>
   </xdr:oneCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
@@ -886,6 +900,9 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="3" max="3" width="24.13"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -3002,6 +3019,528 @@
       </c>
       <c r="I73" s="4">
         <v>4.06273685E7</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="B74" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D74" s="3">
+        <v>10.0007428571429</v>
+      </c>
+      <c r="E74" s="3">
+        <v>15.6413142857143</v>
+      </c>
+      <c r="F74" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G74" s="4">
+        <v>3020970.48571429</v>
+      </c>
+      <c r="H74" s="4">
+        <v>1091278.07142857</v>
+      </c>
+      <c r="I74" s="4">
+        <v>5218774.2</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="B75" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D75" s="3">
+        <v>17.5835428571429</v>
+      </c>
+      <c r="E75" s="3">
+        <v>54.6215428571429</v>
+      </c>
+      <c r="F75" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G75" s="4">
+        <v>4956314.82857143</v>
+      </c>
+      <c r="H75" s="4">
+        <v>1869342.0</v>
+      </c>
+      <c r="I75" s="4">
+        <v>8975610.1</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="B76" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D76" s="3">
+        <v>25.2717714285714</v>
+      </c>
+      <c r="E76" s="3">
+        <v>246.723057142857</v>
+      </c>
+      <c r="F76" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="G76" s="4">
+        <v>6953861.14285714</v>
+      </c>
+      <c r="H76" s="4">
+        <v>2690112.64285714</v>
+      </c>
+      <c r="I76" s="4">
+        <v>1.28385136857143E7</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2">
+        <v>5.0</v>
+      </c>
+      <c r="B77" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D77" s="3">
+        <v>32.4995571428572</v>
+      </c>
+      <c r="E77" s="3">
+        <v>527.987842857143</v>
+      </c>
+      <c r="F77" s="2">
+        <v>14.0</v>
+      </c>
+      <c r="G77" s="4">
+        <v>8661939.02857143</v>
+      </c>
+      <c r="H77" s="4">
+        <v>3294762.84285714</v>
+      </c>
+      <c r="I77" s="4">
+        <v>1.58166926E7</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2">
+        <v>6.0</v>
+      </c>
+      <c r="B78" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D78" s="3">
+        <v>40.4049142857143</v>
+      </c>
+      <c r="E78" s="3">
+        <v>829.436628571429</v>
+      </c>
+      <c r="F78" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="G78" s="4">
+        <v>1.05681339142857E7</v>
+      </c>
+      <c r="H78" s="4">
+        <v>4045741.82857143</v>
+      </c>
+      <c r="I78" s="4">
+        <v>1.94310356571429E7</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2">
+        <v>7.0</v>
+      </c>
+      <c r="B79" s="2">
+        <v>10.0</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D79" s="3">
+        <v>47.4136</v>
+      </c>
+      <c r="E79" s="3">
+        <v>950.6386</v>
+      </c>
+      <c r="F79" s="2">
+        <v>6.0</v>
+      </c>
+      <c r="G79" s="4">
+        <v>1.2280008E7</v>
+      </c>
+      <c r="H79" s="4">
+        <v>4745241.7</v>
+      </c>
+      <c r="I79" s="4">
+        <v>2.27044654E7</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="B80" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D80" s="3">
+        <v>2.61085714285714</v>
+      </c>
+      <c r="E80" s="3">
+        <v>3.09714285714286</v>
+      </c>
+      <c r="F80" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G80" s="4">
+        <v>524526.328571429</v>
+      </c>
+      <c r="H80" s="4">
+        <v>441113.0</v>
+      </c>
+      <c r="I80" s="4">
+        <v>1592668.27142857</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="B81" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D81" s="3">
+        <v>4.25727142857143</v>
+      </c>
+      <c r="E81" s="3">
+        <v>6.1957</v>
+      </c>
+      <c r="F81" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G81" s="4">
+        <v>884535.6</v>
+      </c>
+      <c r="H81" s="4">
+        <v>744848.042857143</v>
+      </c>
+      <c r="I81" s="4">
+        <v>2722272.12857143</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="B82" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D82" s="3">
+        <v>6.1961</v>
+      </c>
+      <c r="E82" s="3">
+        <v>49.0485285714286</v>
+      </c>
+      <c r="F82" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G82" s="4">
+        <v>1295830.07142857</v>
+      </c>
+      <c r="H82" s="4">
+        <v>1084734.9</v>
+      </c>
+      <c r="I82" s="4">
+        <v>4026163.81428571</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2">
+        <v>5.0</v>
+      </c>
+      <c r="B83" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D83" s="3">
+        <v>7.85115714285714</v>
+      </c>
+      <c r="E83" s="3">
+        <v>165.039871428571</v>
+      </c>
+      <c r="F83" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="G83" s="4">
+        <v>1634663.45714286</v>
+      </c>
+      <c r="H83" s="4">
+        <v>1354134.22857143</v>
+      </c>
+      <c r="I83" s="4">
+        <v>5055473.05714286</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2">
+        <v>6.0</v>
+      </c>
+      <c r="B84" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D84" s="3">
+        <v>9.59798571428572</v>
+      </c>
+      <c r="E84" s="3">
+        <v>330.956128571429</v>
+      </c>
+      <c r="F84" s="2">
+        <v>9.0</v>
+      </c>
+      <c r="G84" s="4">
+        <v>2004184.01428571</v>
+      </c>
+      <c r="H84" s="4">
+        <v>1633916.92857143</v>
+      </c>
+      <c r="I84" s="4">
+        <v>6138409.42857143</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2">
+        <v>7.0</v>
+      </c>
+      <c r="B85" s="2">
+        <v>10.0</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D85" s="3">
+        <v>11.4207</v>
+      </c>
+      <c r="E85" s="3">
+        <v>694.0527</v>
+      </c>
+      <c r="F85" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="G85" s="4">
+        <v>2284295.1</v>
+      </c>
+      <c r="H85" s="4">
+        <v>1914095.5</v>
+      </c>
+      <c r="I85" s="4">
+        <v>7141526.3</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="B86" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D86" s="3">
+        <v>9.43737142857143</v>
+      </c>
+      <c r="E86" s="3">
+        <v>14.1913714285714</v>
+      </c>
+      <c r="F86" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G86" s="4">
+        <v>2558790.9</v>
+      </c>
+      <c r="H86" s="4">
+        <v>979289.842857143</v>
+      </c>
+      <c r="I86" s="4">
+        <v>4273248.21428571</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="B87" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D87" s="3">
+        <v>15.9169285714286</v>
+      </c>
+      <c r="E87" s="3">
+        <v>53.3127857142857</v>
+      </c>
+      <c r="F87" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G87" s="4">
+        <v>4259748.94285714</v>
+      </c>
+      <c r="H87" s="4">
+        <v>1710945.52857143</v>
+      </c>
+      <c r="I87" s="4">
+        <v>7468507.77142857</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="B88" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D88" s="3">
+        <v>22.9225285714286</v>
+      </c>
+      <c r="E88" s="3">
+        <v>242.808385714286</v>
+      </c>
+      <c r="F88" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="G88" s="4">
+        <v>5945828.42857143</v>
+      </c>
+      <c r="H88" s="4">
+        <v>2442968.61428571</v>
+      </c>
+      <c r="I88" s="4">
+        <v>1.06853745571429E7</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2">
+        <v>5.0</v>
+      </c>
+      <c r="B89" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D89" s="3">
+        <v>29.1682857142857</v>
+      </c>
+      <c r="E89" s="3">
+        <v>660.299714285714</v>
+      </c>
+      <c r="F89" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="G89" s="4">
+        <v>7424659.48571429</v>
+      </c>
+      <c r="H89" s="4">
+        <v>2999246.32857143</v>
+      </c>
+      <c r="I89" s="4">
+        <v>1.31764169714286E7</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2">
+        <v>6.0</v>
+      </c>
+      <c r="B90" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D90" s="3">
+        <v>36.1905142857143</v>
+      </c>
+      <c r="E90" s="3">
+        <v>826.856942857143</v>
+      </c>
+      <c r="F90" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="G90" s="4">
+        <v>9058220.12857143</v>
+      </c>
+      <c r="H90" s="4">
+        <v>3678640.78571429</v>
+      </c>
+      <c r="I90" s="4">
+        <v>1.62007689428571E7</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2">
+        <v>7.0</v>
+      </c>
+      <c r="B91" s="2">
+        <v>10.0</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D91" s="3">
+        <v>42.3793000000001</v>
+      </c>
+      <c r="E91" s="3">
+        <v>1084.6923</v>
+      </c>
+      <c r="F91" s="2">
+        <v>6.0</v>
+      </c>
+      <c r="G91" s="4">
+        <v>1.05345606E7</v>
+      </c>
+      <c r="H91" s="4">
+        <v>4320872.4</v>
+      </c>
+      <c r="I91" s="4">
+        <v>1.8945501E7</v>
       </c>
     </row>
   </sheetData>
@@ -3010,6 +3549,470 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="O1" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="K2" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="O2" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="P2" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q2" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="R2" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="S2" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="T2" s="7" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="B3" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C3" s="10">
+        <v>14.1426571428571</v>
+      </c>
+      <c r="D3" s="10">
+        <v>21.5619428571429</v>
+      </c>
+      <c r="E3" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="F3" s="12">
+        <v>3916734.14285714</v>
+      </c>
+      <c r="G3" s="12">
+        <v>1015463.02857143</v>
+      </c>
+      <c r="H3" s="12">
+        <v>5894601.0</v>
+      </c>
+      <c r="I3" s="3">
+        <v>5.22294285714286</v>
+      </c>
+      <c r="J3" s="3">
+        <v>5.51208571428571</v>
+      </c>
+      <c r="K3" s="13">
+        <v>0.0</v>
+      </c>
+      <c r="L3" s="4">
+        <v>1136730.55714286</v>
+      </c>
+      <c r="M3" s="4">
+        <v>379174.428571429</v>
+      </c>
+      <c r="N3" s="4">
+        <v>2039514.47142857</v>
+      </c>
+      <c r="O3" s="10">
+        <v>12.6031</v>
+      </c>
+      <c r="P3" s="10">
+        <v>20.0453857142857</v>
+      </c>
+      <c r="Q3" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="R3" s="12">
+        <v>3371983.91428571</v>
+      </c>
+      <c r="S3" s="12">
+        <v>907310.928571429</v>
+      </c>
+      <c r="T3" s="12">
+        <v>4919588.15714286</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="B4" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C4" s="10">
+        <v>31.2545142857143</v>
+      </c>
+      <c r="D4" s="10">
+        <v>51.7892285714286</v>
+      </c>
+      <c r="E4" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="F4" s="12">
+        <v>8051826.25714286</v>
+      </c>
+      <c r="G4" s="12">
+        <v>1749795.42857143</v>
+      </c>
+      <c r="H4" s="12">
+        <v>1.16564129571429E7</v>
+      </c>
+      <c r="I4" s="3">
+        <v>13.6503</v>
+      </c>
+      <c r="J4" s="3">
+        <v>14.9538714285714</v>
+      </c>
+      <c r="K4" s="13">
+        <v>0.0</v>
+      </c>
+      <c r="L4" s="4">
+        <v>3029737.84285714</v>
+      </c>
+      <c r="M4" s="4">
+        <v>644693.557142857</v>
+      </c>
+      <c r="N4" s="4">
+        <v>4559727.28571429</v>
+      </c>
+      <c r="O4" s="10">
+        <v>28.5696</v>
+      </c>
+      <c r="P4" s="10">
+        <v>50.6201714285714</v>
+      </c>
+      <c r="Q4" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="R4" s="12">
+        <v>7145125.6</v>
+      </c>
+      <c r="S4" s="12">
+        <v>1595704.81428571</v>
+      </c>
+      <c r="T4" s="12">
+        <v>1.00673610428571E7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="B5" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C5" s="10">
+        <v>56.2050857142857</v>
+      </c>
+      <c r="D5" s="10">
+        <v>106.5028</v>
+      </c>
+      <c r="E5" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="F5" s="12">
+        <v>1.36750514142857E7</v>
+      </c>
+      <c r="G5" s="12">
+        <v>2530988.0</v>
+      </c>
+      <c r="H5" s="12">
+        <v>1.88339820285714E7</v>
+      </c>
+      <c r="I5" s="3">
+        <v>27.7714285714286</v>
+      </c>
+      <c r="J5" s="3">
+        <v>33.0598571428571</v>
+      </c>
+      <c r="K5" s="13">
+        <v>0.0</v>
+      </c>
+      <c r="L5" s="4">
+        <v>6028459.81428571</v>
+      </c>
+      <c r="M5" s="4">
+        <v>950721.928571429</v>
+      </c>
+      <c r="N5" s="4">
+        <v>8271300.15714286</v>
+      </c>
+      <c r="O5" s="10">
+        <v>50.7758714285714</v>
+      </c>
+      <c r="P5" s="10">
+        <v>107.088157142857</v>
+      </c>
+      <c r="Q5" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="R5" s="12">
+        <v>1.21562619571429E7</v>
+      </c>
+      <c r="S5" s="12">
+        <v>2290298.54285714</v>
+      </c>
+      <c r="T5" s="12">
+        <v>1.64920045428571E7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2">
+        <v>5.0</v>
+      </c>
+      <c r="B6" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C6" s="10">
+        <v>84.5333428571429</v>
+      </c>
+      <c r="D6" s="10">
+        <v>199.343057142857</v>
+      </c>
+      <c r="E6" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="F6" s="12">
+        <v>1.98466040857143E7</v>
+      </c>
+      <c r="G6" s="12">
+        <v>3104847.61428571</v>
+      </c>
+      <c r="H6" s="12">
+        <v>2.60131167857143E7</v>
+      </c>
+      <c r="I6" s="3">
+        <v>44.4713714285714</v>
+      </c>
+      <c r="J6" s="3">
+        <v>55.4899428571429</v>
+      </c>
+      <c r="K6" s="13">
+        <v>0.0</v>
+      </c>
+      <c r="L6" s="4">
+        <v>9584840.87142857</v>
+      </c>
+      <c r="M6" s="4">
+        <v>1193083.75714286</v>
+      </c>
+      <c r="N6" s="4">
+        <v>1.23166056428571E7</v>
+      </c>
+      <c r="O6" s="10">
+        <v>76.4577714285714</v>
+      </c>
+      <c r="P6" s="10">
+        <v>210.815057142857</v>
+      </c>
+      <c r="Q6" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="R6" s="12">
+        <v>1.78130242142857E7</v>
+      </c>
+      <c r="S6" s="12">
+        <v>2816939.05714286</v>
+      </c>
+      <c r="T6" s="12">
+        <v>2.30667877571429E7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2">
+        <v>6.0</v>
+      </c>
+      <c r="B7" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C7" s="10">
+        <v>121.059757142857</v>
+      </c>
+      <c r="D7" s="10">
+        <v>301.900757142857</v>
+      </c>
+      <c r="E7" s="11">
+        <v>1.0</v>
+      </c>
+      <c r="F7" s="12">
+        <v>2.76663663E7</v>
+      </c>
+      <c r="G7" s="12">
+        <v>3820558.84285714</v>
+      </c>
+      <c r="H7" s="12">
+        <v>3.51716087E7</v>
+      </c>
+      <c r="I7" s="3">
+        <v>66.0317428571429</v>
+      </c>
+      <c r="J7" s="3">
+        <v>105.431885714286</v>
+      </c>
+      <c r="K7" s="13">
+        <v>0.0</v>
+      </c>
+      <c r="L7" s="4">
+        <v>1.41415431714286E7</v>
+      </c>
+      <c r="M7" s="4">
+        <v>1442887.1</v>
+      </c>
+      <c r="N7" s="4">
+        <v>1.73448542428571E7</v>
+      </c>
+      <c r="O7" s="10">
+        <v>110.236057142857</v>
+      </c>
+      <c r="P7" s="10">
+        <v>390.583628571429</v>
+      </c>
+      <c r="Q7" s="11">
+        <v>2.0</v>
+      </c>
+      <c r="R7" s="12">
+        <v>2.49468292857143E7</v>
+      </c>
+      <c r="S7" s="12">
+        <v>3462213.42857143</v>
+      </c>
+      <c r="T7" s="12">
+        <v>3.14775868142857E7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2">
+        <v>7.0</v>
+      </c>
+      <c r="B8" s="2">
+        <v>10.0</v>
+      </c>
+      <c r="C8" s="10">
+        <v>167.2031</v>
+      </c>
+      <c r="D8" s="10">
+        <v>417.2621</v>
+      </c>
+      <c r="E8" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="F8" s="12">
+        <v>3.63959479E7</v>
+      </c>
+      <c r="G8" s="12">
+        <v>4487331.2</v>
+      </c>
+      <c r="H8" s="12">
+        <v>4.50571317E7</v>
+      </c>
+      <c r="I8" s="3">
+        <v>93.0603</v>
+      </c>
+      <c r="J8" s="3">
+        <v>297.4273</v>
+      </c>
+      <c r="K8" s="13">
+        <v>1.0</v>
+      </c>
+      <c r="L8" s="4">
+        <v>1.94240914E7</v>
+      </c>
+      <c r="M8" s="4">
+        <v>1695010.6</v>
+      </c>
+      <c r="N8" s="4">
+        <v>2.30804465E7</v>
+      </c>
+      <c r="O8" s="10">
+        <v>149.3563</v>
+      </c>
+      <c r="P8" s="10">
+        <v>554.2473</v>
+      </c>
+      <c r="Q8" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="R8" s="12">
+        <v>3.29426979E7</v>
+      </c>
+      <c r="S8" s="12">
+        <v>4067438.9</v>
+      </c>
+      <c r="T8" s="12">
+        <v>4.06273685E7</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="C1:H1"/>
+    <mergeCell ref="I1:N1"/>
+    <mergeCell ref="O1:T1"/>
+  </mergeCells>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -3593,16 +4596,16 @@
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="5" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="O1" s="5" t="s">
         <v>11</v>
       </c>
       <c r="U1" s="6" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2">
@@ -4924,13 +5927,13 @@
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="5" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I1" s="6" t="s">
         <v>14</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2">
@@ -5951,6 +6954,470 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="O1" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K2" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="O2" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="P2" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q2" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="R2" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="S2" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="T2" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="B3" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C3" s="10">
+        <v>10.0007428571429</v>
+      </c>
+      <c r="D3" s="10">
+        <v>15.6413142857143</v>
+      </c>
+      <c r="E3" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="F3" s="12">
+        <v>3020970.48571429</v>
+      </c>
+      <c r="G3" s="12">
+        <v>1091278.07142857</v>
+      </c>
+      <c r="H3" s="12">
+        <v>5218774.2</v>
+      </c>
+      <c r="I3" s="3">
+        <v>2.61085714285714</v>
+      </c>
+      <c r="J3" s="3">
+        <v>3.09714285714286</v>
+      </c>
+      <c r="K3" s="13">
+        <v>0.0</v>
+      </c>
+      <c r="L3" s="4">
+        <v>524526.328571429</v>
+      </c>
+      <c r="M3" s="4">
+        <v>441113.0</v>
+      </c>
+      <c r="N3" s="4">
+        <v>1592668.27142857</v>
+      </c>
+      <c r="O3" s="10">
+        <v>9.43737142857143</v>
+      </c>
+      <c r="P3" s="10">
+        <v>14.1913714285714</v>
+      </c>
+      <c r="Q3" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="R3" s="12">
+        <v>2558790.9</v>
+      </c>
+      <c r="S3" s="12">
+        <v>979289.842857143</v>
+      </c>
+      <c r="T3" s="12">
+        <v>4273248.21428571</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="B4" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C4" s="10">
+        <v>17.5835428571429</v>
+      </c>
+      <c r="D4" s="10">
+        <v>54.6215428571429</v>
+      </c>
+      <c r="E4" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="F4" s="12">
+        <v>4956314.82857143</v>
+      </c>
+      <c r="G4" s="12">
+        <v>1869342.0</v>
+      </c>
+      <c r="H4" s="12">
+        <v>8975610.1</v>
+      </c>
+      <c r="I4" s="3">
+        <v>4.25727142857143</v>
+      </c>
+      <c r="J4" s="3">
+        <v>6.1957</v>
+      </c>
+      <c r="K4" s="13">
+        <v>0.0</v>
+      </c>
+      <c r="L4" s="4">
+        <v>884535.6</v>
+      </c>
+      <c r="M4" s="4">
+        <v>744848.042857143</v>
+      </c>
+      <c r="N4" s="4">
+        <v>2722272.12857143</v>
+      </c>
+      <c r="O4" s="10">
+        <v>15.9169285714286</v>
+      </c>
+      <c r="P4" s="10">
+        <v>53.3127857142857</v>
+      </c>
+      <c r="Q4" s="11">
+        <v>0.0</v>
+      </c>
+      <c r="R4" s="12">
+        <v>4259748.94285714</v>
+      </c>
+      <c r="S4" s="12">
+        <v>1710945.52857143</v>
+      </c>
+      <c r="T4" s="12">
+        <v>7468507.77142857</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="B5" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C5" s="10">
+        <v>25.2717714285714</v>
+      </c>
+      <c r="D5" s="10">
+        <v>246.723057142857</v>
+      </c>
+      <c r="E5" s="11">
+        <v>2.0</v>
+      </c>
+      <c r="F5" s="12">
+        <v>6953861.14285714</v>
+      </c>
+      <c r="G5" s="12">
+        <v>2690112.64285714</v>
+      </c>
+      <c r="H5" s="12">
+        <v>1.28385136857143E7</v>
+      </c>
+      <c r="I5" s="3">
+        <v>6.1961</v>
+      </c>
+      <c r="J5" s="3">
+        <v>49.0485285714286</v>
+      </c>
+      <c r="K5" s="13">
+        <v>0.0</v>
+      </c>
+      <c r="L5" s="4">
+        <v>1295830.07142857</v>
+      </c>
+      <c r="M5" s="4">
+        <v>1084734.9</v>
+      </c>
+      <c r="N5" s="4">
+        <v>4026163.81428571</v>
+      </c>
+      <c r="O5" s="10">
+        <v>22.9225285714286</v>
+      </c>
+      <c r="P5" s="10">
+        <v>242.808385714286</v>
+      </c>
+      <c r="Q5" s="11">
+        <v>1.0</v>
+      </c>
+      <c r="R5" s="12">
+        <v>5945828.42857143</v>
+      </c>
+      <c r="S5" s="12">
+        <v>2442968.61428571</v>
+      </c>
+      <c r="T5" s="12">
+        <v>1.06853745571429E7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2">
+        <v>5.0</v>
+      </c>
+      <c r="B6" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C6" s="10">
+        <v>32.4995571428572</v>
+      </c>
+      <c r="D6" s="10">
+        <v>527.987842857143</v>
+      </c>
+      <c r="E6" s="11">
+        <v>14.0</v>
+      </c>
+      <c r="F6" s="12">
+        <v>8661939.02857143</v>
+      </c>
+      <c r="G6" s="12">
+        <v>3294762.84285714</v>
+      </c>
+      <c r="H6" s="12">
+        <v>1.58166926E7</v>
+      </c>
+      <c r="I6" s="3">
+        <v>7.85115714285714</v>
+      </c>
+      <c r="J6" s="3">
+        <v>165.039871428571</v>
+      </c>
+      <c r="K6" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="L6" s="4">
+        <v>1634663.45714286</v>
+      </c>
+      <c r="M6" s="4">
+        <v>1354134.22857143</v>
+      </c>
+      <c r="N6" s="4">
+        <v>5055473.05714286</v>
+      </c>
+      <c r="O6" s="10">
+        <v>29.1682857142857</v>
+      </c>
+      <c r="P6" s="10">
+        <v>660.299714285714</v>
+      </c>
+      <c r="Q6" s="11">
+        <v>19.0</v>
+      </c>
+      <c r="R6" s="12">
+        <v>7424659.48571429</v>
+      </c>
+      <c r="S6" s="12">
+        <v>2999246.32857143</v>
+      </c>
+      <c r="T6" s="12">
+        <v>1.31764169714286E7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2">
+        <v>6.0</v>
+      </c>
+      <c r="B7" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C7" s="10">
+        <v>40.4049142857143</v>
+      </c>
+      <c r="D7" s="10">
+        <v>829.436628571429</v>
+      </c>
+      <c r="E7" s="11">
+        <v>29.0</v>
+      </c>
+      <c r="F7" s="12">
+        <v>1.05681339142857E7</v>
+      </c>
+      <c r="G7" s="12">
+        <v>4045741.82857143</v>
+      </c>
+      <c r="H7" s="12">
+        <v>1.94310356571429E7</v>
+      </c>
+      <c r="I7" s="3">
+        <v>9.59798571428572</v>
+      </c>
+      <c r="J7" s="3">
+        <v>330.956128571429</v>
+      </c>
+      <c r="K7" s="13">
+        <v>9.0</v>
+      </c>
+      <c r="L7" s="4">
+        <v>2004184.01428571</v>
+      </c>
+      <c r="M7" s="4">
+        <v>1633916.92857143</v>
+      </c>
+      <c r="N7" s="4">
+        <v>6138409.42857143</v>
+      </c>
+      <c r="O7" s="10">
+        <v>36.1905142857143</v>
+      </c>
+      <c r="P7" s="10">
+        <v>826.856942857143</v>
+      </c>
+      <c r="Q7" s="11">
+        <v>32.0</v>
+      </c>
+      <c r="R7" s="12">
+        <v>9058220.12857143</v>
+      </c>
+      <c r="S7" s="12">
+        <v>3678640.78571429</v>
+      </c>
+      <c r="T7" s="12">
+        <v>1.62007689428571E7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2">
+        <v>7.0</v>
+      </c>
+      <c r="B8" s="2">
+        <v>10.0</v>
+      </c>
+      <c r="C8" s="10">
+        <v>47.4136</v>
+      </c>
+      <c r="D8" s="10">
+        <v>950.6386</v>
+      </c>
+      <c r="E8" s="11">
+        <v>6.0</v>
+      </c>
+      <c r="F8" s="12">
+        <v>1.2280008E7</v>
+      </c>
+      <c r="G8" s="12">
+        <v>4745241.7</v>
+      </c>
+      <c r="H8" s="12">
+        <v>2.27044654E7</v>
+      </c>
+      <c r="I8" s="3">
+        <v>11.4207</v>
+      </c>
+      <c r="J8" s="3">
+        <v>694.0527</v>
+      </c>
+      <c r="K8" s="13">
+        <v>4.0</v>
+      </c>
+      <c r="L8" s="4">
+        <v>2284295.1</v>
+      </c>
+      <c r="M8" s="4">
+        <v>1914095.5</v>
+      </c>
+      <c r="N8" s="4">
+        <v>7141526.3</v>
+      </c>
+      <c r="O8" s="10">
+        <v>42.3793000000001</v>
+      </c>
+      <c r="P8" s="10">
+        <v>1084.6923</v>
+      </c>
+      <c r="Q8" s="11">
+        <v>6.0</v>
+      </c>
+      <c r="R8" s="12">
+        <v>1.05345606E7</v>
+      </c>
+      <c r="S8" s="12">
+        <v>4320872.4</v>
+      </c>
+      <c r="T8" s="12">
+        <v>1.8945501E7</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="C1:H1"/>
+    <mergeCell ref="I1:N1"/>
+    <mergeCell ref="O1:T1"/>
+  </mergeCells>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -5958,22 +7425,22 @@
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="I1" s="14"/>
       <c r="J1" s="14"/>
@@ -34379,7 +35846,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -34709,395 +36176,6 @@
     <mergeCell ref="C1:H1"/>
     <mergeCell ref="I1:N1"/>
   </mergeCells>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2">
-        <v>2.0</v>
-      </c>
-      <c r="B2" s="2">
-        <v>70.0</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" s="3">
-        <v>2.09767142857143</v>
-      </c>
-      <c r="E2" s="3">
-        <v>2.17195714285714</v>
-      </c>
-      <c r="F2" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="G2" s="4">
-        <v>377044.014285714</v>
-      </c>
-      <c r="H2" s="4">
-        <v>287745.4</v>
-      </c>
-      <c r="I2" s="4">
-        <v>1001913.24285714</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2">
-        <v>3.0</v>
-      </c>
-      <c r="B3" s="2">
-        <v>70.0</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="3">
-        <v>6.18141428571429</v>
-      </c>
-      <c r="E3" s="3">
-        <v>6.61898571428571</v>
-      </c>
-      <c r="F3" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="G3" s="4">
-        <v>1163337.74285714</v>
-      </c>
-      <c r="H3" s="4">
-        <v>938139.514285714</v>
-      </c>
-      <c r="I3" s="4">
-        <v>3313619.67142857</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2">
-        <v>4.0</v>
-      </c>
-      <c r="B4" s="2">
-        <v>70.0</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="3">
-        <v>13.0709285714286</v>
-      </c>
-      <c r="E4" s="3">
-        <v>13.7099285714286</v>
-      </c>
-      <c r="F4" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="G4" s="4">
-        <v>2402399.24285714</v>
-      </c>
-      <c r="H4" s="4">
-        <v>1973697.94285714</v>
-      </c>
-      <c r="I4" s="4">
-        <v>7014289.18571429</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2">
-        <v>5.0</v>
-      </c>
-      <c r="B5" s="2">
-        <v>70.0</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="3">
-        <v>22.3752857142857</v>
-      </c>
-      <c r="E5" s="3">
-        <v>23.588</v>
-      </c>
-      <c r="F5" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="G5" s="4">
-        <v>4031384.1</v>
-      </c>
-      <c r="H5" s="4">
-        <v>3356750.21428571</v>
-      </c>
-      <c r="I5" s="4">
-        <v>1.19661421714286E7</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2">
-        <v>6.0</v>
-      </c>
-      <c r="B6" s="2">
-        <v>70.0</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="3">
-        <v>34.2904857142857</v>
-      </c>
-      <c r="E6" s="3">
-        <v>36.5924857142857</v>
-      </c>
-      <c r="F6" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="G6" s="4">
-        <v>6023328.01428571</v>
-      </c>
-      <c r="H6" s="4">
-        <v>5020314.88571429</v>
-      </c>
-      <c r="I6" s="4">
-        <v>1.79053149142857E7</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2">
-        <v>7.0</v>
-      </c>
-      <c r="B7" s="2">
-        <v>10.0</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" s="3">
-        <v>49.4721</v>
-      </c>
-      <c r="E7" s="3">
-        <v>51.9971</v>
-      </c>
-      <c r="F7" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="G7" s="4">
-        <v>8436900.9</v>
-      </c>
-      <c r="H7" s="4">
-        <v>7051733.3</v>
-      </c>
-      <c r="I7" s="4">
-        <v>2.51704999E7</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2">
-        <v>2.0</v>
-      </c>
-      <c r="B8" s="2">
-        <v>70.0</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="3">
-        <v>2.05041428571429</v>
-      </c>
-      <c r="E8" s="3">
-        <v>2.10241428571429</v>
-      </c>
-      <c r="F8" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="G8" s="4">
-        <v>377122.042857143</v>
-      </c>
-      <c r="H8" s="4">
-        <v>287745.4</v>
-      </c>
-      <c r="I8" s="4">
-        <v>1001913.24285714</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2">
-        <v>3.0</v>
-      </c>
-      <c r="B9" s="2">
-        <v>70.0</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" s="3">
-        <v>6.06498571428571</v>
-      </c>
-      <c r="E9" s="3">
-        <v>6.26084285714286</v>
-      </c>
-      <c r="F9" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="G9" s="4">
-        <v>1163463.91428571</v>
-      </c>
-      <c r="H9" s="4">
-        <v>938139.514285714</v>
-      </c>
-      <c r="I9" s="4">
-        <v>3313619.67142857</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2">
-        <v>4.0</v>
-      </c>
-      <c r="B10" s="2">
-        <v>70.0</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="3">
-        <v>12.4792571428571</v>
-      </c>
-      <c r="E10" s="3">
-        <v>12.9208285714286</v>
-      </c>
-      <c r="F10" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="G10" s="4">
-        <v>2402572.94285714</v>
-      </c>
-      <c r="H10" s="4">
-        <v>1973697.94285714</v>
-      </c>
-      <c r="I10" s="4">
-        <v>7014289.18571429</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2">
-        <v>5.0</v>
-      </c>
-      <c r="B11" s="2">
-        <v>70.0</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" s="3">
-        <v>21.9278285714286</v>
-      </c>
-      <c r="E11" s="3">
-        <v>22.7542571428571</v>
-      </c>
-      <c r="F11" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="G11" s="4">
-        <v>4031603.67142857</v>
-      </c>
-      <c r="H11" s="4">
-        <v>3356750.21428571</v>
-      </c>
-      <c r="I11" s="4">
-        <v>1.19661421714286E7</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2">
-        <v>6.0</v>
-      </c>
-      <c r="B12" s="2">
-        <v>70.0</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D12" s="3">
-        <v>33.1871571428571</v>
-      </c>
-      <c r="E12" s="3">
-        <v>34.5567285714286</v>
-      </c>
-      <c r="F12" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="G12" s="4">
-        <v>6023592.48571429</v>
-      </c>
-      <c r="H12" s="4">
-        <v>5020314.88571429</v>
-      </c>
-      <c r="I12" s="4">
-        <v>1.79053149142857E7</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2">
-        <v>7.0</v>
-      </c>
-      <c r="B13" s="2">
-        <v>10.0</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D13" s="3">
-        <v>47.9227</v>
-      </c>
-      <c r="E13" s="3">
-        <v>49.8877</v>
-      </c>
-      <c r="F13" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="G13" s="4">
-        <v>8437210.1</v>
-      </c>
-      <c r="H13" s="4">
-        <v>7051733.3</v>
-      </c>
-      <c r="I13" s="4">
-        <v>2.51704999E7</v>
-      </c>
-    </row>
-  </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -35110,458 +36188,383 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="I1" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="O1" s="5" t="s">
-        <v>34</v>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="K2" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="O2" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="P2" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q2" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="R2" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="S2" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="T2" s="7" t="s">
-        <v>52</v>
+      <c r="A2" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="B2" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" s="3">
+        <v>2.09767142857143</v>
+      </c>
+      <c r="E2" s="3">
+        <v>2.17195714285714</v>
+      </c>
+      <c r="F2" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2" s="4">
+        <v>377044.014285714</v>
+      </c>
+      <c r="H2" s="4">
+        <v>287745.4</v>
+      </c>
+      <c r="I2" s="4">
+        <v>1001913.24285714</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="B3" s="2">
         <v>70.0</v>
       </c>
-      <c r="C3" s="10">
-        <v>14.1426571428571</v>
-      </c>
-      <c r="D3" s="10">
-        <v>21.5619428571429</v>
-      </c>
-      <c r="E3" s="11">
+      <c r="C3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="3">
+        <v>6.18141428571429</v>
+      </c>
+      <c r="E3" s="3">
+        <v>6.61898571428571</v>
+      </c>
+      <c r="F3" s="2">
         <v>0.0</v>
       </c>
-      <c r="F3" s="12">
-        <v>3916734.14285714</v>
-      </c>
-      <c r="G3" s="12">
-        <v>1015463.02857143</v>
-      </c>
-      <c r="H3" s="12">
-        <v>5894601.0</v>
-      </c>
-      <c r="I3" s="3">
-        <v>5.22294285714286</v>
-      </c>
-      <c r="J3" s="3">
-        <v>5.51208571428571</v>
-      </c>
-      <c r="K3" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="L3" s="4">
-        <v>1136730.55714286</v>
-      </c>
-      <c r="M3" s="4">
-        <v>379174.428571429</v>
-      </c>
-      <c r="N3" s="4">
-        <v>2039514.47142857</v>
-      </c>
-      <c r="O3" s="10">
-        <v>12.6031</v>
-      </c>
-      <c r="P3" s="10">
-        <v>20.0453857142857</v>
-      </c>
-      <c r="Q3" s="11">
-        <v>0.0</v>
-      </c>
-      <c r="R3" s="12">
-        <v>3371983.91428571</v>
-      </c>
-      <c r="S3" s="12">
-        <v>907310.928571429</v>
-      </c>
-      <c r="T3" s="12">
-        <v>4919588.15714286</v>
+      <c r="G3" s="4">
+        <v>1163337.74285714</v>
+      </c>
+      <c r="H3" s="4">
+        <v>938139.514285714</v>
+      </c>
+      <c r="I3" s="4">
+        <v>3313619.67142857</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="B4" s="2">
         <v>70.0</v>
       </c>
-      <c r="C4" s="10">
-        <v>31.2545142857143</v>
-      </c>
-      <c r="D4" s="10">
-        <v>51.7892285714286</v>
-      </c>
-      <c r="E4" s="11">
+      <c r="C4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="3">
+        <v>13.0709285714286</v>
+      </c>
+      <c r="E4" s="3">
+        <v>13.7099285714286</v>
+      </c>
+      <c r="F4" s="2">
         <v>0.0</v>
       </c>
-      <c r="F4" s="12">
-        <v>8051826.25714286</v>
-      </c>
-      <c r="G4" s="12">
-        <v>1749795.42857143</v>
-      </c>
-      <c r="H4" s="12">
-        <v>1.16564129571429E7</v>
-      </c>
-      <c r="I4" s="3">
-        <v>13.6503</v>
-      </c>
-      <c r="J4" s="3">
-        <v>14.9538714285714</v>
-      </c>
-      <c r="K4" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="L4" s="4">
-        <v>3029737.84285714</v>
-      </c>
-      <c r="M4" s="4">
-        <v>644693.557142857</v>
-      </c>
-      <c r="N4" s="4">
-        <v>4559727.28571429</v>
-      </c>
-      <c r="O4" s="10">
-        <v>28.5696</v>
-      </c>
-      <c r="P4" s="10">
-        <v>50.6201714285714</v>
-      </c>
-      <c r="Q4" s="11">
-        <v>0.0</v>
-      </c>
-      <c r="R4" s="12">
-        <v>7145125.6</v>
-      </c>
-      <c r="S4" s="12">
-        <v>1595704.81428571</v>
-      </c>
-      <c r="T4" s="12">
-        <v>1.00673610428571E7</v>
+      <c r="G4" s="4">
+        <v>2402399.24285714</v>
+      </c>
+      <c r="H4" s="4">
+        <v>1973697.94285714</v>
+      </c>
+      <c r="I4" s="4">
+        <v>7014289.18571429</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
       <c r="B5" s="2">
         <v>70.0</v>
       </c>
-      <c r="C5" s="10">
-        <v>56.2050857142857</v>
-      </c>
-      <c r="D5" s="10">
-        <v>106.5028</v>
-      </c>
-      <c r="E5" s="11">
+      <c r="C5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="3">
+        <v>22.3752857142857</v>
+      </c>
+      <c r="E5" s="3">
+        <v>23.588</v>
+      </c>
+      <c r="F5" s="2">
         <v>0.0</v>
       </c>
-      <c r="F5" s="12">
-        <v>1.36750514142857E7</v>
-      </c>
-      <c r="G5" s="12">
-        <v>2530988.0</v>
-      </c>
-      <c r="H5" s="12">
-        <v>1.88339820285714E7</v>
-      </c>
-      <c r="I5" s="3">
-        <v>27.7714285714286</v>
-      </c>
-      <c r="J5" s="3">
-        <v>33.0598571428571</v>
-      </c>
-      <c r="K5" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="L5" s="4">
-        <v>6028459.81428571</v>
-      </c>
-      <c r="M5" s="4">
-        <v>950721.928571429</v>
-      </c>
-      <c r="N5" s="4">
-        <v>8271300.15714286</v>
-      </c>
-      <c r="O5" s="10">
-        <v>50.7758714285714</v>
-      </c>
-      <c r="P5" s="10">
-        <v>107.088157142857</v>
-      </c>
-      <c r="Q5" s="11">
-        <v>0.0</v>
-      </c>
-      <c r="R5" s="12">
-        <v>1.21562619571429E7</v>
-      </c>
-      <c r="S5" s="12">
-        <v>2290298.54285714</v>
-      </c>
-      <c r="T5" s="12">
-        <v>1.64920045428571E7</v>
+      <c r="G5" s="4">
+        <v>4031384.1</v>
+      </c>
+      <c r="H5" s="4">
+        <v>3356750.21428571</v>
+      </c>
+      <c r="I5" s="4">
+        <v>1.19661421714286E7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2">
-        <v>5.0</v>
+        <v>6.0</v>
       </c>
       <c r="B6" s="2">
         <v>70.0</v>
       </c>
-      <c r="C6" s="10">
-        <v>84.5333428571429</v>
-      </c>
-      <c r="D6" s="10">
-        <v>199.343057142857</v>
-      </c>
-      <c r="E6" s="11">
+      <c r="C6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="3">
+        <v>34.2904857142857</v>
+      </c>
+      <c r="E6" s="3">
+        <v>36.5924857142857</v>
+      </c>
+      <c r="F6" s="2">
         <v>0.0</v>
       </c>
-      <c r="F6" s="12">
-        <v>1.98466040857143E7</v>
-      </c>
-      <c r="G6" s="12">
-        <v>3104847.61428571</v>
-      </c>
-      <c r="H6" s="12">
-        <v>2.60131167857143E7</v>
-      </c>
-      <c r="I6" s="3">
-        <v>44.4713714285714</v>
-      </c>
-      <c r="J6" s="3">
-        <v>55.4899428571429</v>
-      </c>
-      <c r="K6" s="13">
-        <v>0.0</v>
-      </c>
-      <c r="L6" s="4">
-        <v>9584840.87142857</v>
-      </c>
-      <c r="M6" s="4">
-        <v>1193083.75714286</v>
-      </c>
-      <c r="N6" s="4">
-        <v>1.23166056428571E7</v>
-      </c>
-      <c r="O6" s="10">
-        <v>76.4577714285714</v>
-      </c>
-      <c r="P6" s="10">
-        <v>210.815057142857</v>
-      </c>
-      <c r="Q6" s="11">
-        <v>0.0</v>
-      </c>
-      <c r="R6" s="12">
-        <v>1.78130242142857E7</v>
-      </c>
-      <c r="S6" s="12">
-        <v>2816939.05714286</v>
-      </c>
-      <c r="T6" s="12">
-        <v>2.30667877571429E7</v>
+      <c r="G6" s="4">
+        <v>6023328.01428571</v>
+      </c>
+      <c r="H6" s="4">
+        <v>5020314.88571429</v>
+      </c>
+      <c r="I6" s="4">
+        <v>1.79053149142857E7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2">
-        <v>6.0</v>
+        <v>7.0</v>
       </c>
       <c r="B7" s="2">
-        <v>70.0</v>
-      </c>
-      <c r="C7" s="10">
-        <v>121.059757142857</v>
-      </c>
-      <c r="D7" s="10">
-        <v>301.900757142857</v>
-      </c>
-      <c r="E7" s="11">
-        <v>1.0</v>
-      </c>
-      <c r="F7" s="12">
-        <v>2.76663663E7</v>
-      </c>
-      <c r="G7" s="12">
-        <v>3820558.84285714</v>
-      </c>
-      <c r="H7" s="12">
-        <v>3.51716087E7</v>
-      </c>
-      <c r="I7" s="3">
-        <v>66.0317428571429</v>
-      </c>
-      <c r="J7" s="3">
-        <v>105.431885714286</v>
-      </c>
-      <c r="K7" s="13">
+        <v>10.0</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="3">
+        <v>49.4721</v>
+      </c>
+      <c r="E7" s="3">
+        <v>51.9971</v>
+      </c>
+      <c r="F7" s="2">
         <v>0.0</v>
       </c>
-      <c r="L7" s="4">
-        <v>1.41415431714286E7</v>
-      </c>
-      <c r="M7" s="4">
-        <v>1442887.1</v>
-      </c>
-      <c r="N7" s="4">
-        <v>1.73448542428571E7</v>
-      </c>
-      <c r="O7" s="10">
-        <v>110.236057142857</v>
-      </c>
-      <c r="P7" s="10">
-        <v>390.583628571429</v>
-      </c>
-      <c r="Q7" s="11">
-        <v>2.0</v>
-      </c>
-      <c r="R7" s="12">
-        <v>2.49468292857143E7</v>
-      </c>
-      <c r="S7" s="12">
-        <v>3462213.42857143</v>
-      </c>
-      <c r="T7" s="12">
-        <v>3.14775868142857E7</v>
+      <c r="G7" s="4">
+        <v>8436900.9</v>
+      </c>
+      <c r="H7" s="4">
+        <v>7051733.3</v>
+      </c>
+      <c r="I7" s="4">
+        <v>2.51704999E7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="B8" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="3">
+        <v>2.05041428571429</v>
+      </c>
+      <c r="E8" s="3">
+        <v>2.10241428571429</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G8" s="4">
+        <v>377122.042857143</v>
+      </c>
+      <c r="H8" s="4">
+        <v>287745.4</v>
+      </c>
+      <c r="I8" s="4">
+        <v>1001913.24285714</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="B9" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="3">
+        <v>6.06498571428571</v>
+      </c>
+      <c r="E9" s="3">
+        <v>6.26084285714286</v>
+      </c>
+      <c r="F9" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G9" s="4">
+        <v>1163463.91428571</v>
+      </c>
+      <c r="H9" s="4">
+        <v>938139.514285714</v>
+      </c>
+      <c r="I9" s="4">
+        <v>3313619.67142857</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="B10" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="3">
+        <v>12.4792571428571</v>
+      </c>
+      <c r="E10" s="3">
+        <v>12.9208285714286</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G10" s="4">
+        <v>2402572.94285714</v>
+      </c>
+      <c r="H10" s="4">
+        <v>1973697.94285714</v>
+      </c>
+      <c r="I10" s="4">
+        <v>7014289.18571429</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2">
+        <v>5.0</v>
+      </c>
+      <c r="B11" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" s="3">
+        <v>21.9278285714286</v>
+      </c>
+      <c r="E11" s="3">
+        <v>22.7542571428571</v>
+      </c>
+      <c r="F11" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G11" s="4">
+        <v>4031603.67142857</v>
+      </c>
+      <c r="H11" s="4">
+        <v>3356750.21428571</v>
+      </c>
+      <c r="I11" s="4">
+        <v>1.19661421714286E7</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2">
+        <v>6.0</v>
+      </c>
+      <c r="B12" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12" s="3">
+        <v>33.1871571428571</v>
+      </c>
+      <c r="E12" s="3">
+        <v>34.5567285714286</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G12" s="4">
+        <v>6023592.48571429</v>
+      </c>
+      <c r="H12" s="4">
+        <v>5020314.88571429</v>
+      </c>
+      <c r="I12" s="4">
+        <v>1.79053149142857E7</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2">
         <v>7.0</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B13" s="2">
         <v>10.0</v>
       </c>
-      <c r="C8" s="10">
-        <v>167.2031</v>
-      </c>
-      <c r="D8" s="10">
-        <v>417.2621</v>
-      </c>
-      <c r="E8" s="11">
+      <c r="C13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" s="3">
+        <v>47.9227</v>
+      </c>
+      <c r="E13" s="3">
+        <v>49.8877</v>
+      </c>
+      <c r="F13" s="2">
         <v>0.0</v>
       </c>
-      <c r="F8" s="12">
-        <v>3.63959479E7</v>
-      </c>
-      <c r="G8" s="12">
-        <v>4487331.2</v>
-      </c>
-      <c r="H8" s="12">
-        <v>4.50571317E7</v>
-      </c>
-      <c r="I8" s="3">
-        <v>93.0603</v>
-      </c>
-      <c r="J8" s="3">
-        <v>297.4273</v>
-      </c>
-      <c r="K8" s="13">
-        <v>1.0</v>
-      </c>
-      <c r="L8" s="4">
-        <v>1.94240914E7</v>
-      </c>
-      <c r="M8" s="4">
-        <v>1695010.6</v>
-      </c>
-      <c r="N8" s="4">
-        <v>2.30804465E7</v>
-      </c>
-      <c r="O8" s="10">
-        <v>149.3563</v>
-      </c>
-      <c r="P8" s="10">
-        <v>554.2473</v>
-      </c>
-      <c r="Q8" s="11">
-        <v>0.0</v>
-      </c>
-      <c r="R8" s="12">
-        <v>3.29426979E7</v>
-      </c>
-      <c r="S8" s="12">
-        <v>4067438.9</v>
-      </c>
-      <c r="T8" s="12">
-        <v>4.06273685E7</v>
+      <c r="G13" s="4">
+        <v>8437210.1</v>
+      </c>
+      <c r="H13" s="4">
+        <v>7051733.3</v>
+      </c>
+      <c r="I13" s="4">
+        <v>2.51704999E7</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="C1:H1"/>
-    <mergeCell ref="I1:N1"/>
-    <mergeCell ref="O1:T1"/>
-  </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>